<commit_message>
vault backup: 2026-06-30 20:34:52
</commit_message>
<xml_diff>
--- a/Ashwin_SOTI_6_Week_Sprint .xlsx
+++ b/Ashwin_SOTI_6_Week_Sprint .xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asininite\Documents\ObsidianVault\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC92091-28BD-4BFA-B313-382FBEF7E1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -532,8 +538,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -585,10 +591,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -596,13 +608,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -640,7 +660,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -674,6 +694,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -708,9 +729,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -883,11 +905,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F42"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="23.109375" customWidth="1"/>
+    <col min="4" max="4" width="26.77734375" customWidth="1"/>
+    <col min="5" max="5" width="67.44140625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="50.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -900,14 +928,14 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -920,14 +948,14 @@
       <c r="D2" t="s">
         <v>57</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>89</v>
       </c>
       <c r="F2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -940,14 +968,14 @@
       <c r="D3" t="s">
         <v>57</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3" t="s">
         <v>90</v>
       </c>
       <c r="F3" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -960,14 +988,14 @@
       <c r="D4" t="s">
         <v>58</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="3" t="s">
         <v>91</v>
       </c>
       <c r="F4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -980,14 +1008,14 @@
       <c r="D5" t="s">
         <v>59</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="3" t="s">
         <v>92</v>
       </c>
       <c r="F5" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1000,14 +1028,14 @@
       <c r="D6" t="s">
         <v>60</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="3" t="s">
         <v>93</v>
       </c>
       <c r="F6" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1020,14 +1048,14 @@
       <c r="D7" t="s">
         <v>61</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>94</v>
       </c>
       <c r="F7" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1040,14 +1068,14 @@
       <c r="D8" t="s">
         <v>62</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="3" t="s">
         <v>95</v>
       </c>
       <c r="F8" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -1060,14 +1088,14 @@
       <c r="D9" t="s">
         <v>63</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F9" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1080,14 +1108,14 @@
       <c r="D10" t="s">
         <v>64</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="3" t="s">
         <v>97</v>
       </c>
       <c r="F10" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1100,14 +1128,14 @@
       <c r="D11" t="s">
         <v>64</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="3" t="s">
         <v>98</v>
       </c>
       <c r="F11" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1120,14 +1148,14 @@
       <c r="D12" t="s">
         <v>65</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="3" t="s">
         <v>99</v>
       </c>
       <c r="F12" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1140,14 +1168,14 @@
       <c r="D13" t="s">
         <v>66</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="3" t="s">
         <v>100</v>
       </c>
       <c r="F13" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -1160,14 +1188,14 @@
       <c r="D14" t="s">
         <v>67</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="3" t="s">
         <v>101</v>
       </c>
       <c r="F14" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1180,14 +1208,14 @@
       <c r="D15" t="s">
         <v>68</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="3" t="s">
         <v>102</v>
       </c>
       <c r="F15" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -1200,14 +1228,14 @@
       <c r="D16" t="s">
         <v>69</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="3" t="s">
         <v>103</v>
       </c>
       <c r="F16" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1220,14 +1248,14 @@
       <c r="D17" t="s">
         <v>70</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="3" t="s">
         <v>104</v>
       </c>
       <c r="F17" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1240,14 +1268,14 @@
       <c r="D18" t="s">
         <v>71</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="3" t="s">
         <v>105</v>
       </c>
       <c r="F18" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -1260,14 +1288,14 @@
       <c r="D19" t="s">
         <v>72</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="3" t="s">
         <v>106</v>
       </c>
       <c r="F19" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1280,14 +1308,14 @@
       <c r="D20" t="s">
         <v>73</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="3" t="s">
         <v>107</v>
       </c>
       <c r="F20" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1300,14 +1328,14 @@
       <c r="D21" t="s">
         <v>74</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="3" t="s">
         <v>108</v>
       </c>
       <c r="F21" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -1320,14 +1348,14 @@
       <c r="D22" t="s">
         <v>75</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="3" t="s">
         <v>109</v>
       </c>
       <c r="F22" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -1340,14 +1368,14 @@
       <c r="D23" t="s">
         <v>75</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="3" t="s">
         <v>110</v>
       </c>
       <c r="F23" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1360,14 +1388,14 @@
       <c r="D24" t="s">
         <v>76</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="3" t="s">
         <v>111</v>
       </c>
       <c r="F24" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1380,14 +1408,14 @@
       <c r="D25" t="s">
         <v>77</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="3" t="s">
         <v>112</v>
       </c>
       <c r="F25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -1400,14 +1428,14 @@
       <c r="D26" t="s">
         <v>77</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="3" t="s">
         <v>113</v>
       </c>
       <c r="F26" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -1420,14 +1448,14 @@
       <c r="D27" t="s">
         <v>78</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="3" t="s">
         <v>114</v>
       </c>
       <c r="F27" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -1440,14 +1468,14 @@
       <c r="D28" t="s">
         <v>79</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="3" t="s">
         <v>115</v>
       </c>
       <c r="F28" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -1460,14 +1488,14 @@
       <c r="D29" t="s">
         <v>80</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="3" t="s">
         <v>116</v>
       </c>
       <c r="F29" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1480,14 +1508,14 @@
       <c r="D30" t="s">
         <v>80</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="3" t="s">
         <v>117</v>
       </c>
       <c r="F30" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -1500,14 +1528,14 @@
       <c r="D31" t="s">
         <v>81</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="3" t="s">
         <v>118</v>
       </c>
       <c r="F31" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -1520,14 +1548,14 @@
       <c r="D32" t="s">
         <v>82</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="3" t="s">
         <v>119</v>
       </c>
       <c r="F32" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -1540,14 +1568,14 @@
       <c r="D33" t="s">
         <v>83</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="3" t="s">
         <v>120</v>
       </c>
       <c r="F33" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -1560,14 +1588,14 @@
       <c r="D34" t="s">
         <v>84</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F34" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1580,14 +1608,14 @@
       <c r="D35" t="s">
         <v>85</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E35" s="3" t="s">
         <v>122</v>
       </c>
       <c r="F35" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1600,14 +1628,14 @@
       <c r="D36" t="s">
         <v>86</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E36" s="3" t="s">
         <v>123</v>
       </c>
       <c r="F36" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1620,14 +1648,14 @@
       <c r="D37" t="s">
         <v>86</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="3" t="s">
         <v>124</v>
       </c>
       <c r="F37" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1640,14 +1668,14 @@
       <c r="D38" t="s">
         <v>87</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" s="3" t="s">
         <v>125</v>
       </c>
       <c r="F38" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1660,14 +1688,14 @@
       <c r="D39" t="s">
         <v>87</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" s="3" t="s">
         <v>126</v>
       </c>
       <c r="F39" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1680,14 +1708,14 @@
       <c r="D40" t="s">
         <v>87</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E40" s="3" t="s">
         <v>127</v>
       </c>
       <c r="F40" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1700,14 +1728,14 @@
       <c r="D41" t="s">
         <v>88</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E41" s="3" t="s">
         <v>128</v>
       </c>
       <c r="F41" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -1720,7 +1748,7 @@
       <c r="D42" t="s">
         <v>88</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E42" s="3" t="s">
         <v>129</v>
       </c>
       <c r="F42" t="s">

</xml_diff>

<commit_message>
Recovered corrupted git repository
</commit_message>
<xml_diff>
--- a/Ashwin_SOTI_6_Week_Sprint .xlsx
+++ b/Ashwin_SOTI_6_Week_Sprint .xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asininite\Documents\ObsidianVault\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC92091-28BD-4BFA-B313-382FBEF7E1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -538,8 +532,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -591,16 +585,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -608,21 +596,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -660,7 +640,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -694,7 +674,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -729,10 +708,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -905,17 +883,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="3" max="3" width="23.109375" customWidth="1"/>
-    <col min="4" max="4" width="26.77734375" customWidth="1"/>
-    <col min="5" max="5" width="67.44140625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="50.44140625" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -928,14 +900,14 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -948,14 +920,14 @@
       <c r="D2" t="s">
         <v>57</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" t="s">
         <v>89</v>
       </c>
       <c r="F2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -968,14 +940,14 @@
       <c r="D3" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" t="s">
         <v>90</v>
       </c>
       <c r="F3" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -988,14 +960,14 @@
       <c r="D4" t="s">
         <v>58</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" t="s">
         <v>91</v>
       </c>
       <c r="F4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1008,14 +980,14 @@
       <c r="D5" t="s">
         <v>59</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" t="s">
         <v>92</v>
       </c>
       <c r="F5" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1028,14 +1000,14 @@
       <c r="D6" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" t="s">
         <v>93</v>
       </c>
       <c r="F6" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1048,14 +1020,14 @@
       <c r="D7" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" t="s">
         <v>94</v>
       </c>
       <c r="F7" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1068,14 +1040,14 @@
       <c r="D8" t="s">
         <v>62</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" t="s">
         <v>95</v>
       </c>
       <c r="F8" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -1088,14 +1060,14 @@
       <c r="D9" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" t="s">
         <v>96</v>
       </c>
       <c r="F9" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1108,14 +1080,14 @@
       <c r="D10" t="s">
         <v>64</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" t="s">
         <v>97</v>
       </c>
       <c r="F10" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1128,14 +1100,14 @@
       <c r="D11" t="s">
         <v>64</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" t="s">
         <v>98</v>
       </c>
       <c r="F11" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1148,14 +1120,14 @@
       <c r="D12" t="s">
         <v>65</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" t="s">
         <v>99</v>
       </c>
       <c r="F12" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1168,14 +1140,14 @@
       <c r="D13" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" t="s">
         <v>100</v>
       </c>
       <c r="F13" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -1188,14 +1160,14 @@
       <c r="D14" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" t="s">
         <v>101</v>
       </c>
       <c r="F14" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1208,14 +1180,14 @@
       <c r="D15" t="s">
         <v>68</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" t="s">
         <v>102</v>
       </c>
       <c r="F15" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -1228,14 +1200,14 @@
       <c r="D16" t="s">
         <v>69</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" t="s">
         <v>103</v>
       </c>
       <c r="F16" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1248,14 +1220,14 @@
       <c r="D17" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" t="s">
         <v>104</v>
       </c>
       <c r="F17" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1268,14 +1240,14 @@
       <c r="D18" t="s">
         <v>71</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" t="s">
         <v>105</v>
       </c>
       <c r="F18" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -1288,14 +1260,14 @@
       <c r="D19" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" t="s">
         <v>106</v>
       </c>
       <c r="F19" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1308,14 +1280,14 @@
       <c r="D20" t="s">
         <v>73</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" t="s">
         <v>107</v>
       </c>
       <c r="F20" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1328,14 +1300,14 @@
       <c r="D21" t="s">
         <v>74</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" t="s">
         <v>108</v>
       </c>
       <c r="F21" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -1348,14 +1320,14 @@
       <c r="D22" t="s">
         <v>75</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" t="s">
         <v>109</v>
       </c>
       <c r="F22" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -1368,14 +1340,14 @@
       <c r="D23" t="s">
         <v>75</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" t="s">
         <v>110</v>
       </c>
       <c r="F23" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1388,14 +1360,14 @@
       <c r="D24" t="s">
         <v>76</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" t="s">
         <v>111</v>
       </c>
       <c r="F24" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1408,14 +1380,14 @@
       <c r="D25" t="s">
         <v>77</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" t="s">
         <v>112</v>
       </c>
       <c r="F25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -1428,14 +1400,14 @@
       <c r="D26" t="s">
         <v>77</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" t="s">
         <v>113</v>
       </c>
       <c r="F26" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -1448,14 +1420,14 @@
       <c r="D27" t="s">
         <v>78</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" t="s">
         <v>114</v>
       </c>
       <c r="F27" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -1468,14 +1440,14 @@
       <c r="D28" t="s">
         <v>79</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" t="s">
         <v>115</v>
       </c>
       <c r="F28" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -1488,14 +1460,14 @@
       <c r="D29" t="s">
         <v>80</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" t="s">
         <v>116</v>
       </c>
       <c r="F29" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1508,14 +1480,14 @@
       <c r="D30" t="s">
         <v>80</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" t="s">
         <v>117</v>
       </c>
       <c r="F30" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -1528,14 +1500,14 @@
       <c r="D31" t="s">
         <v>81</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" t="s">
         <v>118</v>
       </c>
       <c r="F31" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -1548,14 +1520,14 @@
       <c r="D32" t="s">
         <v>82</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" t="s">
         <v>119</v>
       </c>
       <c r="F32" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -1568,14 +1540,14 @@
       <c r="D33" t="s">
         <v>83</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" t="s">
         <v>120</v>
       </c>
       <c r="F33" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -1588,14 +1560,14 @@
       <c r="D34" t="s">
         <v>84</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" t="s">
         <v>121</v>
       </c>
       <c r="F34" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1608,14 +1580,14 @@
       <c r="D35" t="s">
         <v>85</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="E35" t="s">
         <v>122</v>
       </c>
       <c r="F35" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1628,14 +1600,14 @@
       <c r="D36" t="s">
         <v>86</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" t="s">
         <v>123</v>
       </c>
       <c r="F36" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1648,14 +1620,14 @@
       <c r="D37" t="s">
         <v>86</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" t="s">
         <v>124</v>
       </c>
       <c r="F37" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1668,14 +1640,14 @@
       <c r="D38" t="s">
         <v>87</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" t="s">
         <v>125</v>
       </c>
       <c r="F38" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1688,14 +1660,14 @@
       <c r="D39" t="s">
         <v>87</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E39" t="s">
         <v>126</v>
       </c>
       <c r="F39" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1708,14 +1680,14 @@
       <c r="D40" t="s">
         <v>87</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" t="s">
         <v>127</v>
       </c>
       <c r="F40" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1728,14 +1700,14 @@
       <c r="D41" t="s">
         <v>88</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" t="s">
         <v>128</v>
       </c>
       <c r="F41" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -1748,7 +1720,7 @@
       <c r="D42" t="s">
         <v>88</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" t="s">
         <v>129</v>
       </c>
       <c r="F42" t="s">

</xml_diff>